<commit_message>
Added CartPageTest and update the framework with singleton design patterns
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\eclipse-workspace\OrangrHRMAUtomation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5EA6F8C-DE0E-4960-83A8-39640357AC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C41B25-FEE4-47EA-A052-75819BDCA91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8097A74F-8D50-48FC-B003-6DDC2ADF1112}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginTest" sheetId="1" r:id="rId1"/>
+    <sheet name="Valid LoginTest" sheetId="1" r:id="rId1"/>
+    <sheet name="Invalid LoginTest" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
   <si>
     <t>Test Scenario</t>
   </si>
@@ -74,6 +75,12 @@
   </si>
   <si>
     <t>faizal789@gmail.com</t>
+  </si>
+  <si>
+    <t>Valid LoginTest_TC_01</t>
+  </si>
+  <si>
+    <t>Valid LoginTest_TC_02</t>
   </si>
 </sst>
 </file>
@@ -493,6 +500,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F73142-EE32-41FA-AF6E-B522C2ABCA7D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{E853D13E-A274-41AF-89CA-AFB8983F816A}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{DAC83865-E228-46A6-8171-808564AE5C11}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{9F61FC4F-C17F-4DE1-BA66-74EFE051D5F3}"/>
+    <hyperlink ref="C3" r:id="rId4" xr:uid="{D40C14C3-DA6C-4FD6-BBEB-2CD8D25138F9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05D448A6-3297-44C6-A315-C54F159197CC}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -546,14 +608,13 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{E853D13E-A274-41AF-89CA-AFB8983F816A}"/>
-    <hyperlink ref="C2" r:id="rId2" xr:uid="{DAC83865-E228-46A6-8171-808564AE5C11}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{9F61FC4F-C17F-4DE1-BA66-74EFE051D5F3}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{2A5B768E-F19E-493D-A4CC-4ABFD8296FD9}"/>
-    <hyperlink ref="C3" r:id="rId5" xr:uid="{D40C14C3-DA6C-4FD6-BBEB-2CD8D25138F9}"/>
-    <hyperlink ref="C4" r:id="rId6" display="Faizal@123" xr:uid="{F5BE906D-A964-4EA1-A137-514D7D0AE01B}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{223AFCB4-72A3-45ED-A42E-771D314976A2}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{4C787B02-46BB-4A25-BD62-771DD92497DA}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{532896E5-985F-44C6-87B9-30FD538578AF}"/>
+    <hyperlink ref="B4" r:id="rId4" xr:uid="{AE9FDCF5-1D57-483C-B6B0-23499E435404}"/>
+    <hyperlink ref="C3" r:id="rId5" xr:uid="{19BA4D65-3BD6-44E9-93D8-B697BEF14AB7}"/>
+    <hyperlink ref="C4" r:id="rId6" display="Faizal@123" xr:uid="{9191E16D-3E18-46AB-A48B-4632C5D2BDAE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>